<commit_message>
Add ASIANENE Stage 2 research note and correct Stage 1 history read
Research note (R1-R21) built from the filing repository, annual reports and
public sources, with tagged citations. History read v2 and model notes correct
the FY17/FY18/FY21 non-cash adjustment description and the FY17 write-back line.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015epyZKZUkmLvmzDXXcj4JD
</commit_message>
<xml_diff>
--- a/research/ASIANENE/ASIANENE_Model_v1.xlsx
+++ b/research/ASIANENE/ASIANENE_Model_v1.xlsx
@@ -156,7 +156,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Contains ESOP charge (Rs.9.2cr FY26; Rs.30.1cr FY21; Rs.29.5cr FY18 per ARs), share of JV profit reversal, unrealised FX and sundry write-offs. FY17-FY18 ESOP charges (Rs.43cr, Rs.29cr) are the reason reported PAT and cash profit diverge in those years.</t>
+          <t xml:space="preserve">Contains the FY26 ESOP charge (Rs.9.2cr), share of JV profit reversal, unrealised FX, and bad-debt write-offs and provisions. The large FY17/FY18/FY21 figures (Rs.43cr/Rs.29cr/Rs.30cr) are mainly receivable write-offs and provisions, not ESOP (audited ESOP expense under Rs.0.5cr in those years).</t>
         </r>
       </text>
     </comment>
@@ -1085,7 +1085,7 @@
     <t xml:space="preserve">FY17 promoter change</t>
   </si>
   <si>
-    <t xml:space="preserve">Oilmax Energy Pvt Ltd (Kapil Garg) acquired control in FY17 via preferential issue (Rs.88.6cr equity raised in FY17, Rs.48cr in FY18). Business re-based from this point; large ESOP charges in FY17-FY18 and FY21 (Rs.43cr, Rs.29cr, Rs.30cr per AR cash-flow notes) depress reported PAT in those years.</t>
+    <t xml:space="preserve">Oilmax Energy Pvt Ltd (Kapil Garg) acquired control in FY17 via preferential issue (Rs.88.6cr equity raised in FY17, Rs.48cr in FY18). Business re-based from this point; large receivable write-offs and provisions in FY17-FY18 and FY21 (non-cash adjustments of Rs.43cr, Rs.29cr, Rs.30cr) depress reported PAT in those years; a Rs.19.2cr payables/ICD write-back is booked as an exceptional gain in FY17.</t>
   </si>
   <si>
     <t xml:space="preserve">FY23 reclassification</t>
@@ -1385,15 +1385,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1405,143 +1405,143 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1553,15 +1553,15 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1569,19 +1569,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1589,19 +1589,19 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1864,18 +1864,18 @@
   <dimension ref="A1:AA211"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="2" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
         <v>28</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>791.0474</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
         <v>29</v>
       </c>
@@ -2118,12 +2118,12 @@
         <v>0.701037828943478</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
         <v>31</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>-0.1147</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
         <v>32</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>33</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>-0.1147</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
         <v>34</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>791.1621</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
         <v>35</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>1.00014499763225</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
         <v>36</v>
       </c>
@@ -2615,7 +2615,7 @@
         <v>1.1548</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>37</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>42.1453</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>38</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>607.6703</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>39</v>
       </c>
@@ -2828,7 +2828,7 @@
         <v>40.1986</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
         <v>40</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>41</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>4.6372</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>42</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>695.6915</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
         <v>43</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>95.3559</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
         <v>29</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>0.442426030132512</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
         <v>44</v>
       </c>
@@ -3338,7 +3338,7 @@
         <v>0.120543851101717</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
         <v>45</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>8.8908</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
         <v>46</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>18.8635</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
         <v>47</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>85.3832</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
         <v>48</v>
       </c>
@@ -3644,7 +3644,7 @@
         <v>10.6512</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
         <v>49</v>
       </c>
@@ -3715,7 +3715,7 @@
         <v>3.5077</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
         <v>50</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>-9.4031</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
         <v>51</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>68.8366</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
         <v>52</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>16.9979</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
         <v>53</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>0.246931138376968</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
         <v>54</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>51.8387</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
         <v>55</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>0.6816</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
         <v>56</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>51.1571</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
         <v>29</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>0.21446664656685</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
         <v>44</v>
       </c>
@@ -4482,7 +4482,7 @@
         <v>0.0646700817169743</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
         <v>57</v>
       </c>
@@ -4575,7 +4575,7 @@
         <v>4.49175</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
         <v>58</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>11.3891245060389</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
         <v>59</v>
       </c>
@@ -4761,7 +4761,7 @@
         <v>5.6146875</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
         <v>60</v>
       </c>
@@ -4832,7 +4832,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
         <v>61</v>
       </c>
@@ -4941,12 +4941,12 @@
         <v>FY30E</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
         <v>63</v>
       </c>
@@ -5017,7 +5017,7 @@
         <v>44.9175</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
         <v>64</v>
       </c>
@@ -5088,7 +5088,7 @@
         <v>53.9924</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
         <v>65</v>
       </c>
@@ -5159,7 +5159,7 @@
         <v>395.2431</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
         <v>66</v>
       </c>
@@ -5252,7 +5252,7 @@
         <v>494.153</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
         <v>67</v>
       </c>
@@ -5323,12 +5323,12 @@
         <v>0.8232</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
         <v>69</v>
       </c>
@@ -5399,7 +5399,7 @@
         <v>72.2426</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
         <v>70</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
         <v>71</v>
       </c>
@@ -5541,7 +5541,7 @@
         <v>-5.0725</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
         <v>72</v>
       </c>
@@ -5612,7 +5612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="11" t="s">
         <v>73</v>
       </c>
@@ -5683,7 +5683,7 @@
         <v>12.3796</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
         <v>74</v>
       </c>
@@ -5776,12 +5776,12 @@
         <v>79.5497</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="s">
         <v>76</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>229.5765</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
         <v>77</v>
       </c>
@@ -5923,7 +5923,7 @@
         <v>35.5735</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="s">
         <v>78</v>
       </c>
@@ -5994,7 +5994,7 @@
         <v>60.7017</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
         <v>79</v>
       </c>
@@ -6065,7 +6065,7 @@
         <v>12.9618</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
         <v>80</v>
       </c>
@@ -6158,7 +6158,7 @@
         <v>338.8135</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
         <v>81</v>
       </c>
@@ -6251,17 +6251,17 @@
         <v>913.3394</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="s">
         <v>84</v>
       </c>
@@ -6332,7 +6332,7 @@
         <v>362.7596</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
         <v>85</v>
       </c>
@@ -6403,7 +6403,7 @@
         <v>248.2026</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="s">
         <v>86</v>
       </c>
@@ -6496,7 +6496,7 @@
         <v>114.557</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
         <v>87</v>
       </c>
@@ -6567,7 +6567,7 @@
         <v>46.1305</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="11" t="s">
         <v>88</v>
       </c>
@@ -6638,7 +6638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
         <v>89</v>
       </c>
@@ -6709,7 +6709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="11" t="s">
         <v>90</v>
       </c>
@@ -6780,7 +6780,7 @@
         <v>11.9357</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
         <v>91</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>13.5488</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="11" t="s">
         <v>92</v>
       </c>
@@ -6922,7 +6922,7 @@
         <v>12.0668</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="s">
         <v>93</v>
       </c>
@@ -7015,12 +7015,12 @@
         <v>198.2388</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="11" t="s">
         <v>95</v>
       </c>
@@ -7091,7 +7091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
         <v>96</v>
       </c>
@@ -7162,7 +7162,7 @@
         <v>0.2925</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="11" t="s">
         <v>97</v>
       </c>
@@ -7233,7 +7233,7 @@
         <v>347.7344</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
         <v>98</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>146.8454</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="11" t="s">
         <v>99</v>
       </c>
@@ -7375,7 +7375,7 @@
         <v>9.7443</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
         <v>100</v>
       </c>
@@ -7446,7 +7446,7 @@
         <v>210.484</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="s">
         <v>101</v>
       </c>
@@ -7539,7 +7539,7 @@
         <v>715.1006</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
         <v>102</v>
       </c>
@@ -7610,7 +7610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="6" t="s">
         <v>103</v>
       </c>
@@ -7703,7 +7703,7 @@
         <v>913.3394</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="27" t="s">
         <v>104</v>
       </c>
@@ -7796,7 +7796,7 @@
         <v>0.205349289316776</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="29" t="s">
         <v>105</v>
       </c>
@@ -7889,7 +7889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
         <v>106</v>
       </c>
@@ -7998,7 +7998,7 @@
         <v>FY30E</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="6" t="s">
         <v>107</v>
       </c>
@@ -8069,12 +8069,12 @@
         <v>68.8366</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="6" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
         <v>109</v>
       </c>
@@ -8145,7 +8145,7 @@
         <v>18.8635</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="11" t="s">
         <v>110</v>
       </c>
@@ -8216,7 +8216,7 @@
         <v>7.4251</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
         <v>111</v>
       </c>
@@ -8287,7 +8287,7 @@
         <v>0.0732</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="11" t="s">
         <v>112</v>
       </c>
@@ -8358,7 +8358,7 @@
         <v>-1.0745</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
         <v>113</v>
       </c>
@@ -8429,7 +8429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="11" t="s">
         <v>114</v>
       </c>
@@ -8500,7 +8500,7 @@
         <v>-4.4949</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
         <v>115</v>
       </c>
@@ -8571,7 +8571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="11" t="s">
         <v>116</v>
       </c>
@@ -8642,7 +8642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
         <v>117</v>
       </c>
@@ -8713,7 +8713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="11" t="s">
         <v>118</v>
       </c>
@@ -8784,7 +8784,7 @@
         <v>0.8695</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
         <v>119</v>
       </c>
@@ -8855,7 +8855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="11" t="s">
         <v>120</v>
       </c>
@@ -8926,7 +8926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
         <v>121</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="11" t="s">
         <v>122</v>
       </c>
@@ -9068,7 +9068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
         <v>123</v>
       </c>
@@ -9139,7 +9139,7 @@
         <v>5.6717</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="6" t="s">
         <v>124</v>
       </c>
@@ -9232,12 +9232,12 @@
         <v>28.8336</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="6" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
         <v>126</v>
       </c>
@@ -9308,7 +9308,7 @@
         <v>19.4056</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="11" t="s">
         <v>96</v>
       </c>
@@ -9379,7 +9379,7 @@
         <v>-0.1147</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
         <v>127</v>
       </c>
@@ -9450,7 +9450,7 @@
         <v>-67.2842</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="11" t="s">
         <v>128</v>
       </c>
@@ -9521,7 +9521,7 @@
         <v>18.8738</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
         <v>129</v>
       </c>
@@ -9592,7 +9592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="6" t="s">
         <v>130</v>
       </c>
@@ -9685,7 +9685,7 @@
         <v>-29.1195</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="6" t="s">
         <v>131</v>
       </c>
@@ -9778,7 +9778,7 @@
         <v>68.5507</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
         <v>132</v>
       </c>
@@ -9849,7 +9849,7 @@
         <v>-15.5655</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="6" t="s">
         <v>133</v>
       </c>
@@ -9942,12 +9942,12 @@
         <v>52.9852</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="6" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
         <v>135</v>
       </c>
@@ -10018,7 +10018,7 @@
         <v>-60.6415</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="11" t="s">
         <v>136</v>
       </c>
@@ -10089,7 +10089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
         <v>112</v>
       </c>
@@ -10160,7 +10160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="11" t="s">
         <v>137</v>
       </c>
@@ -10231,7 +10231,7 @@
         <v>-58.29</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
         <v>138</v>
       </c>
@@ -10302,7 +10302,7 @@
         <v>77.7437</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="11" t="s">
         <v>139</v>
       </c>
@@ -10373,7 +10373,7 @@
         <v>-122.8003</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
         <v>140</v>
       </c>
@@ -10444,7 +10444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="11" t="s">
         <v>141</v>
       </c>
@@ -10515,7 +10515,7 @@
         <v>4.4949</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
         <v>142</v>
       </c>
@@ -10586,7 +10586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="11" t="s">
         <v>143</v>
       </c>
@@ -10657,7 +10657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="6" t="s">
         <v>144</v>
       </c>
@@ -10750,12 +10750,12 @@
         <v>-159.4932</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="6" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="11" t="s">
         <v>146</v>
       </c>
@@ -10826,7 +10826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
         <v>147</v>
       </c>
@@ -10897,7 +10897,7 @@
         <v>96.718</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="11" t="s">
         <v>148</v>
       </c>
@@ -10968,7 +10968,7 @@
         <v>-7.2092</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
         <v>149</v>
       </c>
@@ -11039,7 +11039,7 @@
         <v>44.8918</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="11" t="s">
         <v>150</v>
       </c>
@@ -11110,7 +11110,7 @@
         <v>2.1835</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
         <v>151</v>
       </c>
@@ -11181,7 +11181,7 @@
         <v>-4.424</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="11" t="s">
         <v>152</v>
       </c>
@@ -11252,7 +11252,7 @@
         <v>-7.4251</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
         <v>153</v>
       </c>
@@ -11323,7 +11323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="11" t="s">
         <v>154</v>
       </c>
@@ -11394,7 +11394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
         <v>155</v>
       </c>
@@ -11465,7 +11465,7 @@
         <v>-1.1224</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="6" t="s">
         <v>156</v>
       </c>
@@ -11558,7 +11558,7 @@
         <v>123.6126</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="6" t="s">
         <v>157</v>
       </c>
@@ -11651,7 +11651,7 @@
         <v>17.1046</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
         <v>158</v>
       </c>
@@ -11722,7 +11722,7 @@
         <v>19.9296</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="11" t="s">
         <v>159</v>
       </c>
@@ -11793,7 +11793,7 @@
         <v>71.7139</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="6" t="s">
         <v>160</v>
       </c>
@@ -11886,7 +11886,7 @@
         <v>108.7481</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="27" t="s">
         <v>161</v>
       </c>
@@ -11957,7 +11957,7 @@
         <v>108.7481</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="29" t="s">
         <v>105</v>
       </c>
@@ -12050,7 +12050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
         <v>162</v>
       </c>
@@ -12159,12 +12159,12 @@
         <v>FY30E</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="11" t="s">
         <v>164</v>
       </c>
@@ -12257,7 +12257,7 @@
         <v>97.6702</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
         <v>165</v>
       </c>
@@ -12350,7 +12350,7 @@
         <v>4.4949</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="11" t="s">
         <v>166</v>
       </c>
@@ -12443,7 +12443,7 @@
         <v>2.1835</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
         <v>167</v>
       </c>
@@ -12536,7 +12536,7 @@
         <v>134.4006</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="6" t="s">
         <v>168</v>
       </c>
@@ -12629,12 +12629,12 @@
         <v>238.7492</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="6" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
         <v>170</v>
       </c>
@@ -12727,7 +12727,7 @@
         <v>29.1195</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="11" t="s">
         <v>171</v>
       </c>
@@ -12820,7 +12820,7 @@
         <v>15.5655</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
         <v>172</v>
       </c>
@@ -12913,7 +12913,7 @@
         <v>60.6415</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="11" t="s">
         <v>173</v>
       </c>
@@ -13006,7 +13006,7 @@
         <v>-19.4537</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
         <v>174</v>
       </c>
@@ -13099,7 +13099,7 @@
         <v>122.8003</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="11" t="s">
         <v>175</v>
       </c>
@@ -13192,7 +13192,7 @@
         <v>-0</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
         <v>176</v>
       </c>
@@ -13285,7 +13285,7 @@
         <v>4.424</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="11" t="s">
         <v>177</v>
       </c>
@@ -13378,7 +13378,7 @@
         <v>1.1224</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="6" t="s">
         <v>178</v>
       </c>
@@ -13471,7 +13471,7 @@
         <v>214.2195</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="34" t="s">
         <v>179</v>
       </c>
@@ -13564,7 +13564,7 @@
         <v>-7.65630000000001</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="34" t="s">
         <v>180</v>
       </c>
@@ -13657,7 +13657,7 @@
         <v>126.7443</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="27" t="s">
         <v>181</v>
       </c>
@@ -13750,7 +13750,7 @@
         <v>1.02211668116677</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="3" t="s">
         <v>182</v>
       </c>
@@ -13859,7 +13859,7 @@
         <v>FY30E</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="11" t="s">
         <v>183</v>
       </c>
@@ -13948,7 +13948,7 @@
         <v>0.108501399536867</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="11" t="s">
         <v>184</v>
       </c>
@@ -14037,7 +14037,7 @@
         <v>131.99895448743</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="11" t="s">
         <v>185</v>
       </c>
@@ -14126,7 +14126,7 @@
         <v>209.174064348104</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="11" t="s">
         <v>186</v>
       </c>
@@ -14215,7 +14215,7 @@
         <v>85.8278369286088</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="6" t="s">
         <v>187</v>
       </c>
@@ -14304,7 +14304,7 @@
         <v>123.454728819032</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="3" t="s">
         <v>188</v>
       </c>
@@ -14413,7 +14413,7 @@
         <v>FY30E</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="11" t="s">
         <v>189</v>
       </c>
@@ -14506,7 +14506,7 @@
         <v>494.153</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="11" t="s">
         <v>190</v>
       </c>
@@ -14595,7 +14595,7 @@
         <v>446.4125</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="11" t="s">
         <v>191</v>
       </c>
@@ -14684,7 +14684,7 @@
         <v>0.11459602945706</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="11" t="s">
         <v>192</v>
       </c>
@@ -14773,7 +14773,7 @@
         <v>752.89805</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="11" t="s">
         <v>193</v>
       </c>
@@ -14862,7 +14862,7 @@
         <v>0.0909767705460327</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="11" t="s">
         <v>194</v>
       </c>
@@ -14933,7 +14933,7 @@
         <v>25.1738</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="11" t="s">
         <v>195</v>
       </c>
@@ -15026,7 +15026,7 @@
         <v>158.1181</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="11" t="s">
         <v>196</v>
       </c>
@@ -15119,7 +15119,7 @@
         <v>11.2727</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="11" t="s">
         <v>197</v>
       </c>
@@ -15212,7 +15212,7 @@
         <v>0.118217121331769</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="11" t="s">
         <v>198</v>
       </c>
@@ -15305,7 +15305,7 @@
         <v>0.0228121654629234</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="11" t="s">
         <v>199</v>
       </c>
@@ -15394,7 +15394,7 @@
         <v>0.183933330167282</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="11" t="s">
         <v>200</v>
       </c>
@@ -15483,7 +15483,7 @@
         <v>1.0506700077122</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="11" t="s">
         <v>201</v>
       </c>
@@ -15572,7 +15572,7 @@
         <v>2.26936461024636</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="11" t="s">
         <v>202</v>
       </c>
@@ -15665,12 +15665,12 @@
         <v>3.21475335966284</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="11" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="27" t="s">
         <v>204</v>
       </c>
@@ -15741,7 +15741,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="27" t="s">
         <v>209</v>
       </c>
@@ -15766,11 +15766,11 @@
   <dimension ref="A1:K37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>210</v>
       </c>
@@ -15805,12 +15805,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
         <v>212</v>
       </c>
@@ -15833,7 +15833,7 @@
         <v>632.68</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>29</v>
       </c>
@@ -15858,7 +15858,7 @@
         <v>2.2876740802328</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
         <v>213</v>
       </c>
@@ -15881,7 +15881,7 @@
         <v>158.37</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>29</v>
       </c>
@@ -15906,7 +15906,7 @@
         <v>-0.419017572177996</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>214</v>
       </c>
@@ -15935,7 +15935,7 @@
         <v>791.05</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
         <v>215</v>
       </c>
@@ -15964,7 +15964,7 @@
         <v>0.799797737184754</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
         <v>216</v>
       </c>
@@ -15993,12 +15993,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
         <v>218</v>
       </c>
@@ -16021,7 +16021,7 @@
         <v>101.96</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>219</v>
       </c>
@@ -16044,7 +16044,7 @@
         <v>31.6</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>220</v>
       </c>
@@ -16073,7 +16073,7 @@
         <v>133.56</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>221</v>
       </c>
@@ -16096,7 +16096,7 @@
         <v>18.86</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
         <v>222</v>
       </c>
@@ -16119,7 +16119,7 @@
         <v>8.89</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>223</v>
       </c>
@@ -16142,7 +16142,7 @@
         <v>10.65</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
         <v>224</v>
       </c>
@@ -16165,7 +16165,7 @@
         <v>38.2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
         <v>225</v>
       </c>
@@ -16194,13 +16194,13 @@
         <v>74.74</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B23" s="44" t="n">
@@ -16228,8 +16228,8 @@
         <v>0.161155718530695</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>228</v>
       </c>
       <c r="B24" s="44" t="n">
@@ -16257,8 +16257,8 @@
         <v>0.199532739786576</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>229</v>
       </c>
       <c r="B25" s="44" t="n">
@@ -16286,23 +16286,23 @@
         <v>0.168838885026231</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="27" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
         <v>233</v>
       </c>
       <c r="F31" s="13" t="n">
@@ -16312,8 +16312,8 @@
         <v>299.37</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>234</v>
       </c>
       <c r="F32" s="13" t="n">
@@ -16323,8 +16323,8 @@
         <v>142.96</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
         <v>235</v>
       </c>
       <c r="F33" s="13" t="n">
@@ -16334,8 +16334,8 @@
         <v>264.36</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>236</v>
       </c>
       <c r="F34" s="45" t="n">
@@ -16350,7 +16350,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="27" t="s">
         <v>238</v>
       </c>
@@ -16374,13 +16374,13 @@
   <dimension ref="A2:H22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="4" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="47" t="s">
         <v>239</v>
       </c>
@@ -16391,7 +16391,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="49" t="s">
         <v>241</v>
       </c>
@@ -16403,7 +16403,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="49" t="s">
         <v>243</v>
       </c>
@@ -16412,12 +16412,12 @@
         <v>2043.74625</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D7" s="51" t="s">
         <v>23</v>
       </c>
@@ -16434,12 +16434,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="49" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="49" t="s">
         <v>246</v>
       </c>
@@ -16467,7 +16467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="49" t="s">
         <v>248</v>
       </c>
@@ -16492,7 +16492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="49" t="str">
         <f aca="false">CONCATENATE("-@CMP of Rs.",ROUND($C$2,0),"/share")</f>
         <v>-@CMP of Rs.455/share</v>
@@ -16521,7 +16521,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="54" t="n">
         <v>8</v>
       </c>
@@ -16549,7 +16549,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="54" t="n">
         <v>10</v>
       </c>
@@ -16577,7 +16577,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="54" t="n">
         <v>12</v>
       </c>
@@ -16605,7 +16605,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="27" t="s">
         <v>251</v>
       </c>
@@ -16626,13 +16626,13 @@
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="49" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="1" t="s">
         <v>253</v>
       </c>
       <c r="C18" s="53" t="n">
@@ -16640,8 +16640,8 @@
         <v>39.9503930050765</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="1" t="s">
         <v>254</v>
       </c>
       <c r="C19" s="53" t="n">
@@ -16649,8 +16649,8 @@
         <v>4.1358572142636</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="1" t="s">
         <v>255</v>
       </c>
       <c r="C20" s="53" t="n">
@@ -16682,12 +16682,12 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="120"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="120"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="3" style="1" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
         <v>257</v>
       </c>
@@ -16717,11 +16717,11 @@
         <v>263</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11"/>
       <c r="B5" s="56"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
         <v>264</v>
       </c>
@@ -16799,17 +16799,17 @@
         <v>282</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11"/>
       <c r="B16" s="56"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>283</v>
       </c>
       <c r="B17" s="56"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>284</v>
       </c>
@@ -16832,8 +16832,8 @@
         <v>290</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="13" t="n">
@@ -16855,8 +16855,8 @@
         <v>494.2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="13" t="n">
@@ -16878,8 +16878,8 @@
         <v>398.7</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B21" s="13" t="n">
@@ -16901,8 +16901,8 @@
         <v>277.9</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="13" t="n">
@@ -16924,8 +16924,8 @@
         <v>199.5</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B23" s="13" t="n">
@@ -16947,8 +16947,8 @@
         <v>241.8</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="13" t="n">
@@ -16970,8 +16970,8 @@
         <v>203.4</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B25" s="13" t="n">
@@ -16993,8 +16993,8 @@
         <v>181.5</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B26" s="13" t="n">
@@ -17016,8 +17016,8 @@
         <v>152</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B27" s="13" t="n">
@@ -17039,8 +17039,8 @@
         <v>140.5</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B28" s="13" t="n">
@@ -17062,8 +17062,8 @@
         <v>81.8</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B29" s="13" t="n">
@@ -17085,8 +17085,8 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B30" s="13" t="n">
@@ -17108,8 +17108,8 @@
         <v>37.2</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B31" s="13" t="n">
@@ -17131,8 +17131,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B32" s="13" t="n">
@@ -17154,8 +17154,8 @@
         <v>72.2</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B33" s="13" t="n">
@@ -17177,8 +17177,8 @@
         <v>82.3</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B34" s="13" t="n">
@@ -17200,8 +17200,8 @@
         <v>91.5</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B35" s="13" t="n">
@@ -17223,8 +17223,8 @@
         <v>100.4</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B36" s="13" t="n">
@@ -17246,7 +17246,7 @@
         <v>77.9</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
         <v>291</v>
       </c>
@@ -17284,11 +17284,11 @@
         <v>299</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11"/>
       <c r="B44" s="56"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
         <v>300</v>
       </c>

</xml_diff>